<commit_message>
Reset to 0.5 in all future years
</commit_message>
<xml_diff>
--- a/InputData/trans/FoSfBPPTtC/Fraction of Subsidy for Battery Production Passed Through to Consumers.xlsx
+++ b/InputData/trans/FoSfBPPTtC/Fraction of Subsidy for Battery Production Passed Through to Consumers.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Olivia Ashmoore\Documents\EPS_Models by Region\United States\us-eps\InputData\trans\FoSfBPPTtC\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MeganMahajan\Documents\eps-us\InputData\trans\FoSfBPPTtC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7C9B15B-257A-4BDB-B4D2-0C8D459E3DBA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E1232FB-AC72-4B08-A84C-F862671FD419}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-90" yWindow="-90" windowWidth="19380" windowHeight="10260" activeTab="1" xr2:uid="{DC12087C-9A27-4A43-B4A9-6B3F1E517F08}"/>
+    <workbookView xWindow="38280" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="1" xr2:uid="{DC12087C-9A27-4A43-B4A9-6B3F1E517F08}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -425,17 +425,17 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EF982137-6F01-4109-8226-D4C6F3731BA9}">
   <dimension ref="A1:B8"/>
-  <sheetFormatPr defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="101.26953125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.75">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.75">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>0</v>
       </c>
@@ -443,27 +443,27 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.75">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B4" s="2">
         <v>2023</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.75">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B5" s="2" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.75">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B6" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.75">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B7" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.75">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A8" s="1"/>
     </row>
   </sheetData>
@@ -477,12 +477,12 @@
     <tabColor theme="4" tint="-0.249977111117893"/>
   </sheetPr>
   <dimension ref="A1:AE2"/>
-  <sheetFormatPr defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="21.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:31" x14ac:dyDescent="0.75">
+    <row r="1" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>2</v>
       </c>
@@ -577,15 +577,15 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="2" spans="1:31" ht="29.5" x14ac:dyDescent="0.75">
+    <row r="2" spans="1:31" ht="29" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
         <v>3</v>
       </c>
       <c r="B2">
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="C2">
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="D2">
         <v>0.25</v>
@@ -597,79 +597,79 @@
         <v>0.5</v>
       </c>
       <c r="G2">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="H2">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="I2">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J2">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="K2">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="L2">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="M2">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="N2">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="O2">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="P2">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="Q2">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="R2">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="S2">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="T2">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="U2">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="V2">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="W2">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="X2">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="Y2">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="Z2">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="AA2">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="AB2">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="AC2">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="AD2">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="AE2">
-        <v>0</v>
+        <v>0.5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>